<commit_message>
model train with raw data
</commit_message>
<xml_diff>
--- a/model_results.xlsx
+++ b/model_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mmeliht/Desktop/URL-Phishing-Detection/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFC169C6-DC6F-9046-9E37-0F0773446194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F753AE53-CE8D-8B41-B9C6-66B61ED4DD6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="120">
   <si>
     <t>Model</t>
   </si>
@@ -86,6 +86,300 @@
   </si>
   <si>
     <t>Naive Bayes</t>
+  </si>
+  <si>
+    <t>Feature Reduced</t>
+  </si>
+  <si>
+    <t>Article Features</t>
+  </si>
+  <si>
+    <t>0.997803</t>
+  </si>
+  <si>
+    <t>0.999629</t>
+  </si>
+  <si>
+    <t>0.996161</t>
+  </si>
+  <si>
+    <t>0.997892</t>
+  </si>
+  <si>
+    <t>0.5496</t>
+  </si>
+  <si>
+    <t>0.0146</t>
+  </si>
+  <si>
+    <t>89.53</t>
+  </si>
+  <si>
+    <t>0.998916</t>
+  </si>
+  <si>
+    <t>0.998153</t>
+  </si>
+  <si>
+    <t>0.998228</t>
+  </si>
+  <si>
+    <t>0.999115</t>
+  </si>
+  <si>
+    <t>0.997788</t>
+  </si>
+  <si>
+    <t>0.999515</t>
+  </si>
+  <si>
+    <t>0.996246</t>
+  </si>
+  <si>
+    <t>0.997878</t>
+  </si>
+  <si>
+    <t>0.4039</t>
+  </si>
+  <si>
+    <t>-278.73</t>
+  </si>
+  <si>
+    <t>90.7</t>
+  </si>
+  <si>
+    <t>0.998850</t>
+  </si>
+  <si>
+    <t>0.998174</t>
+  </si>
+  <si>
+    <t>0.998249</t>
+  </si>
+  <si>
+    <t>0.999103</t>
+  </si>
+  <si>
+    <t>0.997535</t>
+  </si>
+  <si>
+    <t>0.999116</t>
+  </si>
+  <si>
+    <t>0.997636</t>
+  </si>
+  <si>
+    <t>0.3191</t>
+  </si>
+  <si>
+    <t>388.94</t>
+  </si>
+  <si>
+    <t>0.998671</t>
+  </si>
+  <si>
+    <t>0.997811</t>
+  </si>
+  <si>
+    <t>0.997901</t>
+  </si>
+  <si>
+    <t>0.998920</t>
+  </si>
+  <si>
+    <t>0.997149</t>
+  </si>
+  <si>
+    <t>0.999514</t>
+  </si>
+  <si>
+    <t>0.995023</t>
+  </si>
+  <si>
+    <t>0.997264</t>
+  </si>
+  <si>
+    <t>0.0055</t>
+  </si>
+  <si>
+    <t>275.80</t>
+  </si>
+  <si>
+    <t>100.0</t>
+  </si>
+  <si>
+    <t>0.998297</t>
+  </si>
+  <si>
+    <t>0.997473</t>
+  </si>
+  <si>
+    <t>0.997575</t>
+  </si>
+  <si>
+    <t>0.998528</t>
+  </si>
+  <si>
+    <t>0.996897</t>
+  </si>
+  <si>
+    <t>0.998034</t>
+  </si>
+  <si>
+    <t>0.996018</t>
+  </si>
+  <si>
+    <t>0.997025</t>
+  </si>
+  <si>
+    <t>0.7607</t>
+  </si>
+  <si>
+    <t>0.0115</t>
+  </si>
+  <si>
+    <t>194.14</t>
+  </si>
+  <si>
+    <t>0.996943</t>
+  </si>
+  <si>
+    <t>0.997120</t>
+  </si>
+  <si>
+    <t>0.997240</t>
+  </si>
+  <si>
+    <t>0.997187</t>
+  </si>
+  <si>
+    <t>0.996184</t>
+  </si>
+  <si>
+    <t>0.999513</t>
+  </si>
+  <si>
+    <t>0.993174</t>
+  </si>
+  <si>
+    <t>0.996334</t>
+  </si>
+  <si>
+    <t>0.0611</t>
+  </si>
+  <si>
+    <t>153.97</t>
+  </si>
+  <si>
+    <t>0.998465</t>
+  </si>
+  <si>
+    <t>0.996502</t>
+  </si>
+  <si>
+    <t>0.996641</t>
+  </si>
+  <si>
+    <t>0.998722</t>
+  </si>
+  <si>
+    <t>0.991656</t>
+  </si>
+  <si>
+    <t>0.996470</t>
+  </si>
+  <si>
+    <t>0.987515</t>
+  </si>
+  <si>
+    <t>0.991972</t>
+  </si>
+  <si>
+    <t>0.0471</t>
+  </si>
+  <si>
+    <t>276.80</t>
+  </si>
+  <si>
+    <t>90.8</t>
+  </si>
+  <si>
+    <t>0.996981</t>
+  </si>
+  <si>
+    <t>0.992062</t>
+  </si>
+  <si>
+    <t>0.992367</t>
+  </si>
+  <si>
+    <t>0.997341</t>
+  </si>
+  <si>
+    <t>0.964959</t>
+  </si>
+  <si>
+    <t>0.992168</t>
+  </si>
+  <si>
+    <t>0.940303</t>
+  </si>
+  <si>
+    <t>0.965539</t>
+  </si>
+  <si>
+    <t>0.0058</t>
+  </si>
+  <si>
+    <t>352.77</t>
+  </si>
+  <si>
+    <t>91.4</t>
+  </si>
+  <si>
+    <t>0.996446</t>
+  </si>
+  <si>
+    <t>0.962601</t>
+  </si>
+  <si>
+    <t>0.962800</t>
+  </si>
+  <si>
+    <t>0.996614</t>
+  </si>
+  <si>
+    <t>0.921292</t>
+  </si>
+  <si>
+    <t>0.993423</t>
+  </si>
+  <si>
+    <t>0.854896</t>
+  </si>
+  <si>
+    <t>0.918968</t>
+  </si>
+  <si>
+    <t>0.0978</t>
+  </si>
+  <si>
+    <t>0.0198</t>
+  </si>
+  <si>
+    <t>383.27</t>
+  </si>
+  <si>
+    <t>0.955784</t>
+  </si>
+  <si>
+    <t>0.922162</t>
+  </si>
+  <si>
+    <t>0.919927</t>
+  </si>
+  <si>
+    <t>0.955716</t>
   </si>
 </sst>
 </file>
@@ -144,10 +438,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -453,431 +756,852 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="12.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B2">
+      <c r="B3" s="2">
         <v>0.99778800000000001</v>
       </c>
-      <c r="C2">
+      <c r="C3" s="2">
         <v>0.99957200000000002</v>
       </c>
-      <c r="D2">
+      <c r="D3" s="2">
         <v>0.99618899999999999</v>
       </c>
-      <c r="E2">
+      <c r="E3" s="2">
         <v>0.99787800000000004</v>
       </c>
-      <c r="F2">
+      <c r="F3" s="2">
         <v>0.42509999999999998</v>
       </c>
-      <c r="G2">
+      <c r="G3" s="2">
         <v>1.2500000000000001E-2</v>
       </c>
-      <c r="H2">
+      <c r="H3" s="2">
         <v>33.92</v>
       </c>
-      <c r="I2">
+      <c r="I3" s="2">
         <v>2.9</v>
       </c>
-      <c r="J2">
+      <c r="J3" s="2">
         <v>0.99891700000000005</v>
       </c>
-      <c r="K2">
+      <c r="K3" s="2">
         <v>0.998108</v>
       </c>
-      <c r="L2">
+      <c r="L3" s="2">
         <v>0.99818600000000002</v>
       </c>
-      <c r="M2">
+      <c r="M3" s="2">
         <v>0.99911000000000005</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B3">
+      <c r="B4" s="2">
         <v>0.99774300000000005</v>
       </c>
-      <c r="C3">
+      <c r="C4" s="2">
         <v>0.99942900000000001</v>
       </c>
-      <c r="D3">
+      <c r="D4" s="2">
         <v>0.99624599999999996</v>
       </c>
-      <c r="E3">
+      <c r="E4" s="2">
         <v>0.99783500000000003</v>
       </c>
-      <c r="F3">
+      <c r="F4" s="2">
         <v>23.046099999999999</v>
       </c>
-      <c r="G3">
+      <c r="G4" s="2">
         <v>0.41710000000000003</v>
       </c>
-      <c r="H3">
+      <c r="H4" s="2">
         <v>3.64</v>
       </c>
-      <c r="I3">
+      <c r="I4" s="2">
         <v>90.9</v>
       </c>
-      <c r="J3">
+      <c r="J4" s="2">
         <v>0.99885800000000002</v>
       </c>
-      <c r="K3">
+      <c r="K4" s="2">
         <v>0.99811099999999997</v>
       </c>
-      <c r="L3">
+      <c r="L4" s="2">
         <v>0.99818899999999999</v>
       </c>
-      <c r="M3">
+      <c r="M4" s="2">
         <v>0.99910200000000005</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B4">
+      <c r="B5" s="2">
         <v>0.99732699999999996</v>
       </c>
-      <c r="C4">
+      <c r="C5" s="2">
         <v>0.99885900000000005</v>
       </c>
-      <c r="D4">
+      <c r="D5" s="2">
         <v>0.99601799999999996</v>
       </c>
-      <c r="E4">
+      <c r="E5" s="2">
         <v>0.99743700000000002</v>
       </c>
-      <c r="F4">
+      <c r="F5" s="2">
         <v>8.9070999999999998</v>
       </c>
-      <c r="G4">
+      <c r="G5" s="2">
         <v>0.316</v>
       </c>
-      <c r="H4">
+      <c r="H5" s="2">
         <v>61.33</v>
       </c>
-      <c r="I4">
+      <c r="I5" s="2">
         <v>2.9</v>
       </c>
-      <c r="J4">
+      <c r="J5" s="2">
         <v>0.99865000000000004</v>
       </c>
-      <c r="K4">
+      <c r="K5" s="2">
         <v>0.99771900000000002</v>
       </c>
-      <c r="L4">
+      <c r="L5" s="2">
         <v>0.99781299999999995</v>
       </c>
-      <c r="M4">
+      <c r="M5" s="2">
         <v>0.998919</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B5">
+      <c r="B6" s="2">
         <v>0.99705999999999995</v>
       </c>
-      <c r="C5">
+      <c r="C6" s="2">
         <v>0.99937200000000004</v>
       </c>
-      <c r="D5">
+      <c r="D6" s="2">
         <v>0.99499400000000005</v>
       </c>
-      <c r="E5">
+      <c r="E6" s="2">
         <v>0.99717800000000001</v>
       </c>
-      <c r="F5">
+      <c r="F6" s="2">
         <v>10.965400000000001</v>
       </c>
-      <c r="G5">
+      <c r="G6" s="2">
         <v>5.5999999999999999E-3</v>
       </c>
-      <c r="H5">
+      <c r="H6" s="2">
         <v>199.89</v>
       </c>
-      <c r="I5">
+      <c r="I6" s="2">
         <v>93.2</v>
       </c>
-      <c r="J5">
+      <c r="J6" s="2">
         <v>0.99809400000000004</v>
       </c>
-      <c r="K5">
+      <c r="K6" s="2">
         <v>0.99734199999999995</v>
       </c>
-      <c r="L5">
+      <c r="L6" s="2">
         <v>0.99744999999999995</v>
       </c>
-      <c r="M5">
+      <c r="M6" s="2">
         <v>0.99836100000000005</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6">
+      <c r="B7" s="2">
         <v>0.99661500000000003</v>
       </c>
-      <c r="C6">
+      <c r="C7" s="2">
         <v>0.99763500000000005</v>
       </c>
-      <c r="D6">
+      <c r="D7" s="2">
         <v>0.99587599999999998</v>
       </c>
-      <c r="E6">
+      <c r="E7" s="2">
         <v>0.99675499999999995</v>
       </c>
-      <c r="F6">
+      <c r="F7" s="2">
         <v>0.60640000000000005</v>
       </c>
-      <c r="G6">
+      <c r="G7" s="2">
         <v>7.7999999999999996E-3</v>
       </c>
-      <c r="H6">
+      <c r="H7" s="2">
         <v>44.98</v>
       </c>
-      <c r="I6">
+      <c r="I7" s="2">
         <v>3.9</v>
       </c>
-      <c r="J6">
+      <c r="J7" s="2">
         <v>0.99665700000000002</v>
       </c>
-      <c r="K6">
+      <c r="K7" s="2">
         <v>0.99702400000000002</v>
       </c>
-      <c r="L6">
+      <c r="L7" s="2">
         <v>0.99714899999999995</v>
       </c>
-      <c r="M6">
+      <c r="M7" s="2">
         <v>0.99708300000000005</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7">
+      <c r="B8" s="2">
         <v>0.99618399999999996</v>
       </c>
-      <c r="C7">
+      <c r="C8" s="2">
         <v>0.99951299999999998</v>
       </c>
-      <c r="D7">
+      <c r="D8" s="2">
         <v>0.993174</v>
       </c>
-      <c r="E7">
+      <c r="E8" s="2">
         <v>0.99633400000000005</v>
       </c>
-      <c r="F7">
+      <c r="F8" s="2">
         <v>29.432200000000002</v>
       </c>
-      <c r="G7">
+      <c r="G8" s="2">
         <v>5.6399999999999999E-2</v>
       </c>
-      <c r="H7">
+      <c r="H8" s="2">
         <v>83.61</v>
       </c>
-      <c r="I7">
+      <c r="I8" s="2">
         <v>3</v>
       </c>
-      <c r="J7">
+      <c r="J8" s="2">
         <v>0.99846500000000005</v>
       </c>
-      <c r="K7">
+      <c r="K8" s="2">
         <v>0.99646000000000001</v>
       </c>
-      <c r="L7">
+      <c r="L8" s="2">
         <v>0.99660099999999996</v>
       </c>
-      <c r="M7">
+      <c r="M8" s="2">
         <v>0.99871200000000004</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B8">
+      <c r="B9" s="2">
         <v>0.99170000000000003</v>
       </c>
-      <c r="C8">
+      <c r="C9" s="2">
         <v>0.99675499999999995</v>
       </c>
-      <c r="D8">
+      <c r="D9" s="2">
         <v>0.98731500000000005</v>
       </c>
-      <c r="E8">
+      <c r="E9" s="2">
         <v>0.99201300000000003</v>
       </c>
-      <c r="F8">
+      <c r="F9" s="2">
         <v>2.5399999999999999E-2</v>
       </c>
-      <c r="G8">
+      <c r="G9" s="2">
         <v>8.3930000000000007</v>
       </c>
-      <c r="H8">
+      <c r="H9" s="2">
         <v>121.12</v>
       </c>
-      <c r="I8">
+      <c r="I9" s="2">
         <v>93.5</v>
       </c>
-      <c r="J8">
+      <c r="J9" s="2">
         <v>0.996861</v>
       </c>
-      <c r="K8">
+      <c r="K9" s="2">
         <v>0.99175899999999995</v>
       </c>
-      <c r="L8">
+      <c r="L9" s="2">
         <v>0.99207400000000001</v>
       </c>
-      <c r="M8">
+      <c r="M9" s="2">
         <v>0.99722900000000003</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B9">
+      <c r="B10" s="2">
         <v>0.942272</v>
       </c>
-      <c r="C9">
+      <c r="C10" s="2">
         <v>0.99368500000000004</v>
       </c>
-      <c r="D9">
+      <c r="D10" s="2">
         <v>0.89511099999999999</v>
       </c>
-      <c r="E9">
+      <c r="E10" s="2">
         <v>0.94182600000000005</v>
       </c>
-      <c r="F9">
+      <c r="F10" s="2">
         <v>0.62919999999999998</v>
       </c>
-      <c r="G9">
+      <c r="G10" s="2">
         <v>2.8E-3</v>
       </c>
-      <c r="H9">
+      <c r="H10" s="2">
         <v>184.2</v>
       </c>
-      <c r="I9">
+      <c r="I10" s="2">
         <v>92.2</v>
       </c>
-      <c r="J9">
+      <c r="J10" s="2">
         <v>0.99528399999999995</v>
       </c>
-      <c r="K9">
+      <c r="K10" s="2">
         <v>0.94375600000000004</v>
       </c>
-      <c r="L9">
+      <c r="L10" s="2">
         <v>0.94340199999999996</v>
       </c>
-      <c r="M9">
+      <c r="M10" s="2">
         <v>0.99591499999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B10">
+      <c r="B11" s="2">
         <v>0.920713</v>
       </c>
-      <c r="C10">
+      <c r="C11" s="2">
         <v>0.995448</v>
       </c>
-      <c r="D10">
+      <c r="D11" s="2">
         <v>0.852024</v>
       </c>
-      <c r="E10">
+      <c r="E11" s="2">
         <v>0.91816799999999998</v>
       </c>
-      <c r="F10">
+      <c r="F11" s="2">
         <v>5.79E-2</v>
       </c>
-      <c r="G10">
+      <c r="G11" s="2">
         <v>1.11E-2</v>
       </c>
-      <c r="H10">
+      <c r="H11" s="2">
         <v>143.5</v>
       </c>
-      <c r="I10">
+      <c r="I11" s="2">
         <v>4</v>
       </c>
-      <c r="J10">
+      <c r="J11" s="2">
         <v>0.95711800000000002</v>
       </c>
-      <c r="K10">
+      <c r="K11" s="2">
         <v>0.92149300000000001</v>
       </c>
-      <c r="L10">
+      <c r="L11" s="2">
         <v>0.91904300000000005</v>
       </c>
-      <c r="M10">
+      <c r="M11" s="2">
         <v>0.95690799999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I15" s="3">
+        <v>46266</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16" s="4">
+        <v>258065</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" s="4">
+        <v>103564</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I17" s="3">
+        <v>46149</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" s="4">
+        <v>246667</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="I19" s="3">
+        <v>46214</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F20" s="4">
+        <v>378264</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I20" s="3">
+        <v>46266</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G21" s="4">
+        <v>106202</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F22" s="4">
+        <v>14686</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I23" s="3">
+        <v>46180</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>